<commit_message>
feat(web): update COA crop with Tesseract.js, fix excel import columns & date parsing
</commit_message>
<xml_diff>
--- a/三合一單網頁架機伺服器/台積電槽車barcode三合一單-範本.xlsx
+++ b/三合一單網頁架機伺服器/台積電槽車barcode三合一單-範本.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GOOGLE ANGET\三合一單自動產生器\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GOOGLE ANGET\三合一單網頁架機伺服器\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>槽號</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -132,27 +132,15 @@
     <t>E29</t>
   </si>
   <si>
-    <t>26814E29J1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>15P5</t>
   </si>
   <si>
     <t>E44</t>
   </si>
   <si>
-    <t>26814E44J1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>E318</t>
   </si>
   <si>
-    <t>26814E3181</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>15P6</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -160,29 +148,38 @@
     <t>E319</t>
   </si>
   <si>
-    <t>26813E3191</t>
-  </si>
-  <si>
     <t>15P6</t>
   </si>
   <si>
     <t>E315</t>
   </si>
   <si>
-    <t>26813E3151</t>
-  </si>
-  <si>
     <t>15P5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>E320</t>
-  </si>
-  <si>
-    <t>26814E3201</t>
-  </si>
-  <si>
-    <t>18P1</t>
+    <t>26826E3181</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>26826E3091</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>26826E3081</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>26826E3051</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>26826E3021</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>18P3B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -595,44 +592,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>99784</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>117708</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>2874581</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>689428</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="圖片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5333998" y="2839137"/>
-          <a:ext cx="8244869" cy="4109577"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
@@ -694,7 +653,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1031,18 +990,18 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="1" max="1" width="6.625" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="42.21875" customWidth="1"/>
-    <col min="15" max="15" width="48.88671875" customWidth="1"/>
-    <col min="17" max="17" width="24.44140625" customWidth="1"/>
+    <col min="3" max="3" width="20.125" customWidth="1"/>
+    <col min="4" max="4" width="16.875" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="42.25" customWidth="1"/>
+    <col min="15" max="15" width="48.875" customWidth="1"/>
+    <col min="17" max="17" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>10</v>
       </c>
@@ -1061,7 +1020,7 @@
       <c r="N1" s="27"/>
       <c r="O1" s="27"/>
     </row>
-    <row r="2" spans="1:17" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1097,7 +1056,7 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="14"/>
       <c r="C4" s="16"/>
       <c r="D4" s="18"/>
@@ -1142,7 +1101,7 @@
       <c r="N5" s="26"/>
       <c r="O5" s="26"/>
     </row>
-    <row r="6" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="14"/>
       <c r="C6" s="20"/>
       <c r="D6" s="18"/>
@@ -1187,7 +1146,7 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
     </row>
-    <row r="8" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="14"/>
       <c r="C8" s="22"/>
       <c r="D8" s="18"/>
@@ -1232,7 +1191,7 @@
       <c r="N9" s="26"/>
       <c r="O9" s="26"/>
     </row>
-    <row r="10" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="14"/>
       <c r="C10" s="16"/>
       <c r="D10" s="18"/>
@@ -1280,7 +1239,7 @@
       <c r="N11" s="24"/>
       <c r="O11" s="24"/>
     </row>
-    <row r="12" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="14"/>
       <c r="C12" s="16"/>
       <c r="D12" s="18"/>
@@ -1299,7 +1258,7 @@
       <c r="N12" s="24"/>
       <c r="O12" s="24"/>
     </row>
-    <row r="13" spans="1:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>3</v>
       </c>
@@ -1333,7 +1292,7 @@
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="15" spans="1:17" ht="28.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" ht="27.75" x14ac:dyDescent="0.25">
       <c r="B15" s="14"/>
       <c r="C15" s="16"/>
       <c r="D15" s="18"/>
@@ -1342,12 +1301,12 @@
         <v>626206E3191</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>8</v>
       </c>
@@ -1356,7 +1315,7 @@
         <v>||4L12C53161||5E319||626206E3191||375970680||E1550156A</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E19" s="2" t="s">
         <v>12</v>
       </c>
@@ -1404,10 +1363,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="工作表2"/>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11.75" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -1421,7 +1383,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1429,80 +1391,66 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
         <v>24</v>
       </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1515,7 +1463,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="工作表3"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>